<commit_message>
docs: social media planning
I have completed the first three posts and they are already uploaded. I have also planned several more for next week.
</commit_message>
<xml_diff>
--- a/docs/Social Media Planning.xlsx
+++ b/docs/Social Media Planning.xlsx
@@ -1,27 +1,39 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="29628"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="29725"/>
   <workbookPr/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\anita\Downloads\"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\celia\Downloads\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{3A721FBE-801D-4127-A5CF-001E916B7F22}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{1F3AD812-1877-493C-AC1C-93E7B10FB847}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-110" yWindow="-110" windowWidth="19420" windowHeight="10300" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="12456" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="Planning" sheetId="1" r:id="rId1"/>
   </sheets>
-  <calcPr calcId="0"/>
-  <fileRecoveryPr repairLoad="1"/>
+  <calcPr calcId="191029"/>
+  <extLst>
+    <ext xmlns:xcalcf="http://schemas.microsoft.com/office/spreadsheetml/2018/calcfeatures" uri="{B58B0392-4F1F-4190-BB64-5DF3571DCE5F}">
+      <xcalcf:calcFeatures>
+        <xcalcf:feature name="microsoft.com:RD"/>
+        <xcalcf:feature name="microsoft.com:Single"/>
+        <xcalcf:feature name="microsoft.com:FV"/>
+        <xcalcf:feature name="microsoft.com:CNMTM"/>
+        <xcalcf:feature name="microsoft.com:LET_WF"/>
+        <xcalcf:feature name="microsoft.com:LAMBDA_WF"/>
+        <xcalcf:feature name="microsoft.com:ARRAYTEXT_WF"/>
+      </xcalcf:calcFeatures>
+    </ext>
+  </extLst>
 </workbook>
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="12" uniqueCount="12">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="39" uniqueCount="29">
   <si>
     <t>ID Publicación (Canva/Drive)</t>
   </si>
@@ -57,13 +69,64 @@
   </si>
   <si>
     <t>https://www.instagram.com/p/DVLM8XxCHBb/?igsh=Z3RqejNjenJzcjZn</t>
+  </si>
+  <si>
+    <t>ST-002</t>
+  </si>
+  <si>
+    <t>Corrección presentación</t>
+  </si>
+  <si>
+    <t>Instagram, tiktok</t>
+  </si>
+  <si>
+    <t>Publicado</t>
+  </si>
+  <si>
+    <t>ST-003</t>
+  </si>
+  <si>
+    <t>¿Quiénes somos?</t>
+  </si>
+  <si>
+    <t>https://www.instagram.com/p/DVadPnDiC55/?igsh=MWkwMzgyc214dW1nMg==</t>
+  </si>
+  <si>
+    <t>https://www.instagram.com/p/DVbOx_LiEQw/?igsh=azFpamx3OG1lOWE5</t>
+  </si>
+  <si>
+    <t>ST-004</t>
+  </si>
+  <si>
+    <t>Conversaciones</t>
+  </si>
+  <si>
+    <t>ST-005</t>
+  </si>
+  <si>
+    <t>Muestra mockups</t>
+  </si>
+  <si>
+    <t>ST-006</t>
+  </si>
+  <si>
+    <t>Búsqueda usuarios pilotos</t>
+  </si>
+  <si>
+    <t>ST-007</t>
+  </si>
+  <si>
+    <t>Video kill-opener</t>
+  </si>
+  <si>
+    <t xml:space="preserve">https://www.instagram.com/p/DVdwzwjiMCV/?igsh=MWhmengzZ2I2ajRnOQ== </t>
   </si>
 </sst>
 </file>
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:x16r2="http://schemas.microsoft.com/office/spreadsheetml/2015/02/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="x14ac x16r2 xr">
-  <fonts count="3" x14ac:knownFonts="1">
+  <fonts count="4" x14ac:knownFonts="1">
     <font>
       <sz val="10"/>
       <color rgb="FF000000"/>
@@ -81,6 +144,14 @@
       <sz val="10"/>
       <color theme="10"/>
       <name val="Arial"/>
+      <scheme val="minor"/>
+    </font>
+    <font>
+      <u/>
+      <sz val="10"/>
+      <color rgb="FF000000"/>
+      <name val="Arial"/>
+      <family val="2"/>
       <scheme val="minor"/>
     </font>
   </fonts>
@@ -105,12 +176,15 @@
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
     <xf numFmtId="0" fontId="2" fillId="0" borderId="0" applyNumberFormat="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
   </cellStyleXfs>
-  <cellXfs count="5">
+  <cellXfs count="8">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="0" applyFont="1"/>
     <xf numFmtId="14" fontId="1" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1"/>
     <xf numFmtId="20" fontId="1" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1"/>
     <xf numFmtId="0" fontId="2" fillId="0" borderId="0" xfId="1"/>
+    <xf numFmtId="14" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1"/>
+    <xf numFmtId="20" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1"/>
+    <xf numFmtId="0" fontId="3" fillId="0" borderId="0" xfId="0" applyFont="1"/>
   </cellXfs>
   <cellStyles count="2">
     <cellStyle name="Hipervínculo" xfId="1" builtinId="8"/>
@@ -330,8 +404,8 @@
   <sheetPr>
     <outlinePr summaryBelow="0" summaryRight="0"/>
   </sheetPr>
-  <dimension ref="A1:G6"/>
-  <sheetFormatPr baseColWidth="10" defaultColWidth="12.6328125" defaultRowHeight="15.75" customHeight="1" x14ac:dyDescent="0.25"/>
+  <dimension ref="A1:G8"/>
+  <sheetFormatPr baseColWidth="10" defaultColWidth="12.6640625" defaultRowHeight="15.75" customHeight="1" x14ac:dyDescent="0.25"/>
   <sheetData>
     <row r="1" spans="1:7" ht="15.75" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A1" s="1" t="s">
@@ -373,32 +447,144 @@
         <v>8</v>
       </c>
       <c r="F2" s="1" t="s">
-        <v>9</v>
+        <v>15</v>
       </c>
       <c r="G2" s="4" t="s">
         <v>11</v>
       </c>
     </row>
     <row r="3" spans="1:7" ht="15.75" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="C3" s="2"/>
-      <c r="D3" s="3"/>
+      <c r="A3" t="s">
+        <v>12</v>
+      </c>
+      <c r="B3" t="s">
+        <v>13</v>
+      </c>
+      <c r="C3" s="2">
+        <v>46084</v>
+      </c>
+      <c r="D3" s="3">
+        <v>0.33333333333333331</v>
+      </c>
+      <c r="E3" t="s">
+        <v>14</v>
+      </c>
+      <c r="F3" t="s">
+        <v>15</v>
+      </c>
+      <c r="G3" s="4" t="s">
+        <v>18</v>
+      </c>
     </row>
     <row r="4" spans="1:7" ht="15.75" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="C4" s="2"/>
-      <c r="D4" s="3"/>
+      <c r="A4" t="s">
+        <v>16</v>
+      </c>
+      <c r="B4" t="s">
+        <v>17</v>
+      </c>
+      <c r="C4" s="2">
+        <v>46084</v>
+      </c>
+      <c r="D4" s="3">
+        <v>0.64583333333333337</v>
+      </c>
+      <c r="E4" t="s">
+        <v>14</v>
+      </c>
+      <c r="F4" t="s">
+        <v>15</v>
+      </c>
+      <c r="G4" s="4" t="s">
+        <v>19</v>
+      </c>
     </row>
     <row r="5" spans="1:7" ht="15.75" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="C5" s="2"/>
-      <c r="D5" s="3"/>
+      <c r="A5" t="s">
+        <v>20</v>
+      </c>
+      <c r="B5" t="s">
+        <v>21</v>
+      </c>
+      <c r="C5" s="2">
+        <v>46085</v>
+      </c>
+      <c r="D5" s="3">
+        <v>0.64583333333333337</v>
+      </c>
+      <c r="E5" t="s">
+        <v>14</v>
+      </c>
+      <c r="F5" t="s">
+        <v>15</v>
+      </c>
+      <c r="G5" s="4" t="s">
+        <v>28</v>
+      </c>
     </row>
     <row r="6" spans="1:7" ht="15.75" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="C6" s="2"/>
-      <c r="D6" s="3"/>
+      <c r="A6" t="s">
+        <v>22</v>
+      </c>
+      <c r="B6" t="s">
+        <v>23</v>
+      </c>
+      <c r="C6" s="2">
+        <v>46089</v>
+      </c>
+      <c r="D6" s="3">
+        <v>0.6875</v>
+      </c>
+      <c r="E6" t="s">
+        <v>14</v>
+      </c>
+      <c r="F6" t="s">
+        <v>9</v>
+      </c>
+      <c r="G6" s="7"/>
+    </row>
+    <row r="7" spans="1:7" ht="15.75" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A7" t="s">
+        <v>24</v>
+      </c>
+      <c r="B7" t="s">
+        <v>25</v>
+      </c>
+      <c r="C7" s="5">
+        <v>46090</v>
+      </c>
+      <c r="D7" s="6">
+        <v>0.64583333333333337</v>
+      </c>
+      <c r="E7" t="s">
+        <v>14</v>
+      </c>
+      <c r="F7" t="s">
+        <v>9</v>
+      </c>
+    </row>
+    <row r="8" spans="1:7" ht="15.75" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A8" t="s">
+        <v>26</v>
+      </c>
+      <c r="B8" t="s">
+        <v>27</v>
+      </c>
+      <c r="E8" t="s">
+        <v>14</v>
+      </c>
+      <c r="F8" t="s">
+        <v>9</v>
+      </c>
     </row>
   </sheetData>
   <hyperlinks>
     <hyperlink ref="G2" r:id="rId1" xr:uid="{82FDF14A-527F-4210-A0F6-A0120B1C0ADA}"/>
+    <hyperlink ref="G3" r:id="rId2" xr:uid="{E6359CF6-9B8E-4FF8-BD3D-1E68F301CFA9}"/>
+    <hyperlink ref="G4" r:id="rId3" xr:uid="{E3B74509-A1AD-42C0-B3B0-8A6C7E19F983}"/>
+    <hyperlink ref="G5" r:id="rId4" xr:uid="{B46BB8F9-550D-4CAB-A89C-8AFC7E1FA438}"/>
   </hyperlinks>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
+  <pageSetup paperSize="9" orientation="portrait" r:id="rId5"/>
 </worksheet>
 </file>
</xml_diff>